<commit_message>
Added RDF data schemes and visual schemes for economy-table06, fixed xlsx-spreadsheet
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table06.xlsx
+++ b/sources/table_normalization/xlsx/economy-table06.xlsx
@@ -192,12 +192,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="4"/>
-      <color theme="0"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -284,12 +278,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="4"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color indexed="16"/>
       <name val="Arial Unicode MS"/>
@@ -312,6 +300,19 @@
       <color rgb="FFFF0000"/>
       <name val="Arial Unicode MS"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="4"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="5">
@@ -382,7 +383,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -414,39 +415,39 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -455,46 +456,46 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="3" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
@@ -512,12 +513,13 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Заголовок 1" xfId="1" builtinId="16"/>
@@ -1119,25 +1121,25 @@
       <c r="B6" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="49" t="s">
+      <c r="C6" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="D6" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="49" t="s">
+      <c r="E6" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="50" t="s">
+      <c r="F6" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="49" t="s">
+      <c r="G6" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="50" t="s">
+      <c r="H6" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="49" t="s">
+      <c r="I6" s="53" t="s">
         <v>13</v>
       </c>
       <c r="J6" s="52" t="s">
@@ -2915,18 +2917,18 @@
       <c r="L58" s="37"/>
     </row>
     <row r="59" spans="1:12" ht="15" customHeight="1">
-      <c r="A59" s="51" t="s">
+      <c r="A59" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="B59" s="53"/>
-      <c r="C59" s="54"/>
-      <c r="D59" s="55"/>
-      <c r="E59" s="54"/>
-      <c r="F59" s="55"/>
-      <c r="G59" s="54"/>
-      <c r="H59" s="55"/>
-      <c r="I59" s="54"/>
-      <c r="J59" s="55"/>
+      <c r="B59" s="54"/>
+      <c r="C59" s="51"/>
+      <c r="D59" s="51"/>
+      <c r="E59" s="51"/>
+      <c r="F59" s="51"/>
+      <c r="G59" s="51"/>
+      <c r="H59" s="51"/>
+      <c r="I59" s="51"/>
+      <c r="J59" s="51"/>
       <c r="K59" s="37"/>
       <c r="L59" s="37"/>
     </row>
@@ -3141,9 +3143,9 @@
     <hyperlink ref="A2:B2" location="Contents!A1" display="Back to contents"/>
   </hyperlinks>
   <pageMargins left="0.196850393700787" right="0.196850393700787" top="0.196850393700787" bottom="0.196850393700787" header="0.39370078740157499" footer="0.39370078740157499"/>
-  <pageSetup paperSize="9" scale="32" orientation="portrait" horizontalDpi="300"/>
+  <pageSetup paperSize="9" scale="32" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>